<commit_message>
Update leaves.xlsx from Google Sheet
</commit_message>
<xml_diff>
--- a/data/leaves.xlsx
+++ b/data/leaves.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6344" uniqueCount="1206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6346" uniqueCount="1208">
   <si>
     <t>leave_id</t>
   </si>
@@ -3631,6 +3631,12 @@
   </si>
   <si>
     <t>LV-685</t>
+  </si>
+  <si>
+    <t>LV-686</t>
+  </si>
+  <si>
+    <t>محمد صبحي محمد احمد</t>
   </si>
 </sst>
 </file>
@@ -29201,7 +29207,7 @@
       <c r="F665" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="G665" s="1">
+      <c r="G665" s="4">
         <v>0.0</v>
       </c>
       <c r="H665" s="4" t="s">
@@ -29829,64 +29835,184 @@
       </c>
     </row>
     <row r="682" ht="14.25" customHeight="1">
-      <c r="C682" s="11"/>
-      <c r="I682" s="12"/>
-      <c r="J682" s="12"/>
+      <c r="A682" s="1" t="s">
+        <v>1206</v>
+      </c>
+      <c r="B682" s="7">
+        <v>28798.0</v>
+      </c>
+      <c r="C682" s="8">
+        <v>28798.0</v>
+      </c>
+      <c r="D682" s="4" t="s">
+        <v>1207</v>
+      </c>
+      <c r="E682" s="1"/>
+      <c r="F682" s="1"/>
+      <c r="G682" s="4"/>
+      <c r="H682" s="4"/>
+      <c r="I682" s="9">
+        <v>46301.0</v>
+      </c>
+      <c r="J682" s="9">
+        <v>46332.0</v>
+      </c>
+      <c r="K682" s="4"/>
+      <c r="N682" s="4"/>
     </row>
     <row r="683" ht="14.25" customHeight="1">
-      <c r="C683" s="11"/>
-      <c r="I683" s="12"/>
-      <c r="J683" s="12"/>
+      <c r="A683" s="1"/>
+      <c r="B683" s="7"/>
+      <c r="C683" s="8"/>
+      <c r="D683" s="4"/>
+      <c r="E683" s="1"/>
+      <c r="F683" s="1"/>
+      <c r="G683" s="4"/>
+      <c r="H683" s="4"/>
+      <c r="I683" s="9"/>
+      <c r="J683" s="9"/>
+      <c r="K683" s="4"/>
+      <c r="N683" s="4"/>
     </row>
     <row r="684" ht="14.25" customHeight="1">
-      <c r="C684" s="11"/>
-      <c r="I684" s="12"/>
-      <c r="J684" s="12"/>
+      <c r="A684" s="1"/>
+      <c r="B684" s="7"/>
+      <c r="C684" s="8"/>
+      <c r="D684" s="4"/>
+      <c r="E684" s="1"/>
+      <c r="F684" s="1"/>
+      <c r="G684" s="4"/>
+      <c r="H684" s="4"/>
+      <c r="I684" s="9"/>
+      <c r="J684" s="9"/>
+      <c r="K684" s="4"/>
+      <c r="N684" s="4"/>
     </row>
     <row r="685" ht="14.25" customHeight="1">
-      <c r="C685" s="11"/>
-      <c r="I685" s="12"/>
-      <c r="J685" s="12"/>
+      <c r="A685" s="1"/>
+      <c r="B685" s="7"/>
+      <c r="C685" s="8"/>
+      <c r="D685" s="4"/>
+      <c r="E685" s="1"/>
+      <c r="F685" s="1"/>
+      <c r="G685" s="4"/>
+      <c r="H685" s="4"/>
+      <c r="I685" s="9"/>
+      <c r="J685" s="9"/>
+      <c r="K685" s="4"/>
+      <c r="N685" s="4"/>
     </row>
     <row r="686" ht="14.25" customHeight="1">
-      <c r="C686" s="11"/>
-      <c r="I686" s="12"/>
-      <c r="J686" s="12"/>
+      <c r="A686" s="1"/>
+      <c r="B686" s="7"/>
+      <c r="C686" s="8"/>
+      <c r="D686" s="4"/>
+      <c r="E686" s="1"/>
+      <c r="F686" s="1"/>
+      <c r="G686" s="4"/>
+      <c r="H686" s="4"/>
+      <c r="I686" s="9"/>
+      <c r="J686" s="9"/>
+      <c r="K686" s="4"/>
+      <c r="N686" s="4"/>
     </row>
     <row r="687" ht="14.25" customHeight="1">
-      <c r="C687" s="11"/>
-      <c r="I687" s="12"/>
-      <c r="J687" s="12"/>
+      <c r="A687" s="1"/>
+      <c r="B687" s="7"/>
+      <c r="C687" s="8"/>
+      <c r="D687" s="4"/>
+      <c r="E687" s="1"/>
+      <c r="F687" s="1"/>
+      <c r="G687" s="4"/>
+      <c r="H687" s="4"/>
+      <c r="I687" s="9"/>
+      <c r="J687" s="9"/>
+      <c r="K687" s="4"/>
+      <c r="N687" s="4"/>
     </row>
     <row r="688" ht="14.25" customHeight="1">
-      <c r="C688" s="11"/>
-      <c r="I688" s="12"/>
-      <c r="J688" s="12"/>
+      <c r="A688" s="1"/>
+      <c r="B688" s="7"/>
+      <c r="C688" s="8"/>
+      <c r="D688" s="4"/>
+      <c r="E688" s="1"/>
+      <c r="F688" s="1"/>
+      <c r="G688" s="4"/>
+      <c r="H688" s="4"/>
+      <c r="I688" s="9"/>
+      <c r="J688" s="9"/>
+      <c r="K688" s="4"/>
+      <c r="N688" s="4"/>
     </row>
     <row r="689" ht="14.25" customHeight="1">
-      <c r="C689" s="11"/>
-      <c r="I689" s="12"/>
-      <c r="J689" s="12"/>
+      <c r="A689" s="1"/>
+      <c r="B689" s="7"/>
+      <c r="C689" s="8"/>
+      <c r="D689" s="4"/>
+      <c r="E689" s="1"/>
+      <c r="F689" s="1"/>
+      <c r="G689" s="4"/>
+      <c r="H689" s="4"/>
+      <c r="I689" s="9"/>
+      <c r="J689" s="9"/>
+      <c r="K689" s="4"/>
+      <c r="N689" s="4"/>
     </row>
     <row r="690" ht="14.25" customHeight="1">
-      <c r="C690" s="11"/>
-      <c r="I690" s="12"/>
-      <c r="J690" s="12"/>
+      <c r="A690" s="1"/>
+      <c r="B690" s="7"/>
+      <c r="C690" s="8"/>
+      <c r="D690" s="4"/>
+      <c r="E690" s="1"/>
+      <c r="F690" s="1"/>
+      <c r="G690" s="4"/>
+      <c r="H690" s="4"/>
+      <c r="I690" s="9"/>
+      <c r="J690" s="9"/>
+      <c r="K690" s="4"/>
+      <c r="N690" s="4"/>
     </row>
     <row r="691" ht="14.25" customHeight="1">
-      <c r="C691" s="11"/>
-      <c r="I691" s="12"/>
-      <c r="J691" s="12"/>
+      <c r="A691" s="1"/>
+      <c r="B691" s="7"/>
+      <c r="C691" s="8"/>
+      <c r="D691" s="4"/>
+      <c r="E691" s="1"/>
+      <c r="F691" s="1"/>
+      <c r="G691" s="4"/>
+      <c r="H691" s="4"/>
+      <c r="I691" s="9"/>
+      <c r="J691" s="9"/>
+      <c r="K691" s="4"/>
+      <c r="N691" s="4"/>
     </row>
     <row r="692" ht="14.25" customHeight="1">
-      <c r="C692" s="11"/>
-      <c r="I692" s="12"/>
-      <c r="J692" s="12"/>
+      <c r="A692" s="1"/>
+      <c r="B692" s="7"/>
+      <c r="C692" s="8"/>
+      <c r="D692" s="4"/>
+      <c r="E692" s="1"/>
+      <c r="F692" s="1"/>
+      <c r="G692" s="4"/>
+      <c r="H692" s="4"/>
+      <c r="I692" s="9"/>
+      <c r="J692" s="9"/>
+      <c r="K692" s="4"/>
+      <c r="N692" s="4"/>
     </row>
     <row r="693" ht="14.25" customHeight="1">
-      <c r="C693" s="11"/>
-      <c r="I693" s="12"/>
-      <c r="J693" s="12"/>
+      <c r="A693" s="1"/>
+      <c r="B693" s="7"/>
+      <c r="C693" s="8"/>
+      <c r="D693" s="4"/>
+      <c r="E693" s="1"/>
+      <c r="F693" s="1"/>
+      <c r="G693" s="4"/>
+      <c r="H693" s="4"/>
+      <c r="I693" s="9"/>
+      <c r="J693" s="9"/>
+      <c r="K693" s="4"/>
+      <c r="N693" s="4"/>
     </row>
     <row r="694" ht="14.25" customHeight="1">
       <c r="C694" s="11"/>

</xml_diff>